<commit_message>
fixed LACV no NSs exp1 Trvittatus
</commit_message>
<xml_diff>
--- a/2025_10_06_LACV_50N_no_NSs_exp1/data/2025_10_09_LACV_50N_no_NSs_exp1_tidy.xlsx
+++ b/2025_10_06_LACV_50N_no_NSs_exp1/data/2025_10_09_LACV_50N_no_NSs_exp1_tidy.xlsx
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Trvittatus</t>
+          <t>Trivittatus</t>
         </is>
       </c>
       <c r="E54">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Trvittatus</t>
+          <t>Trivittatus</t>
         </is>
       </c>
       <c r="E108">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Trvittatus</t>
+          <t>Trivittatus</t>
         </is>
       </c>
       <c r="E162">

</xml_diff>